<commit_message>
Add Blackstone account section to June 15 report
Ticket #220546 (ODP/Blackstone - Bus Patrol) now appears under its own
Blackstone section with Bronze band badge.

https://claude.ai/code/session_013dMemYx7zhR2dYYuRXw4Mw
</commit_message>
<xml_diff>
--- a/CS_Daily_Incident_Report_20260615.xlsx
+++ b/CS_Daily_Incident_Report_20260615.xlsx
@@ -1700,7 +1700,7 @@
       </c>
       <c r="B12" s="10" t="inlineStr">
         <is>
-          <t>CoreStack (Internal)</t>
+          <t>Blackstone</t>
         </is>
       </c>
       <c r="C12" s="11" t="inlineStr">
@@ -5920,7 +5920,7 @@
       </c>
       <c r="B9" s="10" t="inlineStr">
         <is>
-          <t>CoreStack (Internal)</t>
+          <t>Blackstone</t>
         </is>
       </c>
       <c r="C9" s="11" t="inlineStr">
@@ -11143,7 +11143,7 @@
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>CoreStack (Internal)</t>
+          <t>Blackstone</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">

</xml_diff>